<commit_message>
modify the dup mach
</commit_message>
<xml_diff>
--- a/results/gcd_progress.xlsx
+++ b/results/gcd_progress.xlsx
@@ -611,7 +611,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>[0, 1, 2, 3]</t>
+          <t>[0, 1, 2, 3, 4]</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>[0]</t>
+          <t>[0, 4]</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>[0, 1, 2, 3]</t>
+          <t>[0, 1, 2, 3, 4]</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -2113,7 +2113,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>[4]</t>
+          <t>[0, 4]</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -3686,7 +3686,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>[0, 1, 2, 3]</t>
+          <t>[0, 1, 2, 3, 4]</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -3951,7 +3951,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>[0, 1, 2, 3]</t>
+          <t>[0, 1, 2, 3, 4]</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -4004,7 +4004,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>[0, 1, 2, 3]</t>
+          <t>[0, 1, 2, 3, 4]</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">

</xml_diff>